<commit_message>
feat: Desarrollo del modulo reportes
</commit_message>
<xml_diff>
--- a/User.xlsx
+++ b/User.xlsx
@@ -1,27 +1,150 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SIPeIP\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{62F0F557-F4F1-425D-9977-9E7FCF30E8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="20370" yWindow="-2205" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
+  <si>
+    <t>Usuario</t>
+  </si>
+  <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>Entidad</t>
+  </si>
+  <si>
+    <t>Carlos Andrade</t>
+  </si>
+  <si>
+    <t>Administrador Global</t>
+  </si>
+  <si>
+    <t>Secretaría Nacional de Planificación</t>
+  </si>
+  <si>
+    <t>Laura Mendoza</t>
+  </si>
+  <si>
+    <t>Administrador del Sistema</t>
+  </si>
+  <si>
+    <t>María Fernández</t>
+  </si>
+  <si>
+    <t>Administradora Institucional</t>
+  </si>
+  <si>
+    <t>Ministerio de Transporte y Obras Públicas</t>
+  </si>
+  <si>
+    <t>Jorge Herrera</t>
+  </si>
+  <si>
+    <t>Director de Planificación</t>
+  </si>
+  <si>
+    <t>Andrea Paredes</t>
+  </si>
+  <si>
+    <t>Analista de Planificación</t>
+  </si>
+  <si>
+    <t>Luis Morales</t>
+  </si>
+  <si>
+    <t>Director de Inversión Pública</t>
+  </si>
+  <si>
+    <t>Diana Cevallos</t>
+  </si>
+  <si>
+    <t>Analista de Inversión Pública</t>
+  </si>
+  <si>
+    <t>Pablo Sánchez</t>
+  </si>
+  <si>
+    <t>Auditor Institucional</t>
+  </si>
+  <si>
+    <t>Verónica Castillo</t>
+  </si>
+  <si>
+    <t>Consulta Institucional</t>
+  </si>
+  <si>
+    <t>Fernando Torres</t>
+  </si>
+  <si>
+    <t>Ministerio de Salud Pública</t>
+  </si>
+  <si>
+    <t>Gabriela Vega</t>
+  </si>
+  <si>
+    <t>Ricardo Salazar</t>
+  </si>
+  <si>
+    <t>Ministerio de Educación</t>
+  </si>
+  <si>
+    <t>Daniela Ruiz</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Admin.123</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -49,8 +172,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +460,222 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="D4:G22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="2"/>
+    <col min="4" max="4" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="26.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(PND): Se agrega la gestion completo y pantallas laterales
</commit_message>
<xml_diff>
--- a/User.xlsx
+++ b/User.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SIPeIP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{62F0F557-F4F1-425D-9977-9E7FCF30E8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E86A593-37EF-4BC5-A5B7-126035073EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-2205" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -172,12 +172,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -464,12 +463,10 @@
   <dimension ref="D4:G22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="9.140625" style="2"/>
-    <col min="4" max="4" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="2"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+    <col min="6" max="6" width="34.28515625" customWidth="1"/>
+    <col min="7" max="7" width="38.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="4:7" x14ac:dyDescent="0.25">
@@ -487,190 +484,190 @@
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
+      <c r="E6" s="2"/>
+      <c r="F6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3" t="s">
+      <c r="E10" s="2"/>
+      <c r="F10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3" t="s">
+      <c r="E11" s="2"/>
+      <c r="F11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3" t="s">
+      <c r="E12" s="2"/>
+      <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="13" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3" t="s">
+      <c r="E13" s="2"/>
+      <c r="F13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3" t="s">
+      <c r="E14" s="2"/>
+      <c r="F14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3" t="s">
+      <c r="E15" s="2"/>
+      <c r="F15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3" t="s">
+      <c r="E16" s="2"/>
+      <c r="F16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3" t="s">
+      <c r="E19" s="2"/>
+      <c r="F19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3" t="s">
+      <c r="E20" s="2"/>
+      <c r="F20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3" t="s">
+      <c r="E21" s="2"/>
+      <c r="F21" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3" t="s">
+      <c r="E22" s="2"/>
+      <c r="F22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" s="2" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>